<commit_message>
feat: consolida pipeline e relatórios pós-comentários
</commit_message>
<xml_diff>
--- a/02-Execucao/05-Comentarios_Gestor/01-Coleta_LimeSurvey/20260716-relacao_respostas_796352.xlsx
+++ b/02-Execucao/05-Comentarios_Gestor/01-Coleta_LimeSurvey/20260716-relacao_respostas_796352.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F93"/>
+  <dimension ref="A1:F94"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -447,10 +447,10 @@
         <v>UENF</v>
       </c>
       <c r="C3" t="str">
-        <v>07/07/2026 08:25:13</v>
+        <v>17/07/2026 09:18:47</v>
       </c>
       <c r="D3" t="str">
-        <v>nao</v>
+        <v>sim</v>
       </c>
       <c r="E3" t="str">
         <v/>
@@ -1907,10 +1907,10 @@
         <v>IRM</v>
       </c>
       <c r="C76" t="str">
-        <v>15/07/2026 13:08:29</v>
+        <v>16/07/2026 12:33:45</v>
       </c>
       <c r="D76" t="str">
-        <v>nao</v>
+        <v>sim</v>
       </c>
       <c r="E76" t="str">
         <v>https://www.tcerj.tc.br/limesurvey-novo/index.php/admin/responses/sa/actionDownloadfiles/surveyid/796352/sResponseId/79</v>
@@ -2259,9 +2259,29 @@
         <v>https://www.tcerj.tc.br/limesurvey-novo/index.php/admin/responses/sa/viewquexmlpdf/surveyid/796352/id/96/browselang/</v>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>97</v>
+      </c>
+      <c r="B94" t="str">
+        <v>SETUR</v>
+      </c>
+      <c r="C94" t="str">
+        <v>16/07/2026 12:33:25</v>
+      </c>
+      <c r="D94" t="str">
+        <v>sim</v>
+      </c>
+      <c r="E94" t="str">
+        <v>https://www.tcerj.tc.br/limesurvey-novo/index.php/admin/responses/sa/actionDownloadfiles/surveyid/796352/sResponseId/97</v>
+      </c>
+      <c r="F94" t="str">
+        <v>https://www.tcerj.tc.br/limesurvey-novo/index.php/admin/responses/sa/viewquexmlpdf/surveyid/796352/id/97/browselang/</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F93"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F94"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>